<commit_message>
Prototipo final v1.1: guardrail de atribución, prompt one-shot, robustez, pytest, CLI y README
</commit_message>
<xml_diff>
--- a/outputs/metrics/resultados_finales.xlsx
+++ b/outputs/metrics/resultados_finales.xlsx
@@ -4233,7 +4233,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>2026-10-21T06:34:08</t>
+          <t>2026-10-21T06:41:25</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
         </is>
       </c>
       <c r="B358">
-        <f>============================= 7 passed in 3.08s ===============================</f>
+        <f>============================= 7 passed in 3.02s ===============================</f>
         <v/>
       </c>
     </row>

</xml_diff>